<commit_message>
chore: update week 4 data files and corresponding import spreadsheets
</commit_message>
<xml_diff>
--- a/public/data/week-4b_wayground_import.xlsx
+++ b/public/data/week-4b_wayground_import.xlsx
@@ -585,7 +585,7 @@
     <row r="3" ht="97.5" customHeight="1" s="17">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>หน้าที่หลักของซอฟต์แวร์ Web Server เช่น Nginx ในระบบเครือข่ายคือข้อใด?</t>
+          <t>หน้าที่หลักของ Firewall ในระบบคอมพิวเตอร์และเครือข่ายคือข้อใด?</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
@@ -595,22 +595,22 @@
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>เชื่อมต่อสายไฟอินเทอร์เน็ตเข้ามายังอาคาร</t>
+          <t>เพิ่มความเร็วการเชื่อมต่ออินเทอร์เน็ตของเครื่องลูกข่าย</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>รับส่งแพ็กเกจ HTTP Request และคืนผลลัพธ์เป็นหน้าเว็บเพจ (HTTP Response)</t>
+          <t>ป้องกันระบบจากการบุกรุกโดยกรองข้อมูลการเชื่อมต่อตามกฎที่กำหนด</t>
         </is>
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
-          <t>แจกจ่ายหมายเลข IP Address ให้แก่เครื่องลูกข่ายโดยอัตโนมัติ</t>
+          <t>ลบประวัติการท่องเว็บของผู้ใช้อัตโนมัติในทุกๆ วัน</t>
         </is>
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>ล้างหน้าจอระบบเพื่อลบประวัติการควบคุมระบบทั้งหมด</t>
+          <t>บีบอัดขนาดไฟล์ข้อมูลและโปรแกรมระบบลินุกซ์ทั้งหมด</t>
         </is>
       </c>
       <c r="G3" s="10" t="n"/>
@@ -626,7 +626,7 @@
     <row r="4" ht="12.75" customHeight="1" s="17">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>ช่องทางพอร์ตมาตรฐานในการรับส่งข้อมูลบริการเว็บไซต์ธรรมดา (HTTP) และเว็บแบบเข้ารหัสปลอดภัย (HTTPS) คือพอร์ตหมายเลขใดตามลำดับ?</t>
+          <t>UFW (Uncomplicated Firewall) บนระบบปฏิบัติการลินุกซ์มีลักษณะการทำงานแบบใด?</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
@@ -636,22 +636,22 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>พอร์ต 22 และ พอร์ต 80</t>
+          <t>เป็นโปรแกรมจัดการฐานข้อมูลที่ถูกอัปเกรดจาก MySQL</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>พอร์ต 80 และ พอร์ต 443</t>
+          <t>เป็นตัวครอบการทำงาน (Frontend) ของ iptables เพื่อให้ใช้งานได้ง่ายขึ้น</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>พอร์ต 443 และ พอร์ต 8006</t>
+          <t>เป็นโปรแกรมตรวจจับและกำจัดมัลแวร์และไวรัสบนเครือข่าย</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>พอร์ต 80 และ พอร์ต 8080</t>
+          <t>เป็นโปรโตคอลหลักในการแจกจ่ายไอพีแอดเดรสแก่เครื่องโฮสต์</t>
         </is>
       </c>
       <c r="G4" s="10" t="n"/>
@@ -659,14 +659,14 @@
         <v>2</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J4" s="12" t="n"/>
     </row>
     <row r="5" ht="12.75" customHeight="1" s="17">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>โปรโตคอล SSH (Secure Shell) ซึ่งใช้ควบคุมเซิร์ฟเวอร์ระยะไกลแบบปลอดภัยทางคอนโซล ทำงานอยู่บนช่องพอร์ตมาตรฐานใด?</t>
+          <t>หากสั่งเปิดทำงาน UFW (sudo ufw enable) โดยที่ยังไม่ได้ตั้งค่าอนุญาตพอร์ต SSH จะเกิดผลกระทบอย่างไร?</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
@@ -676,37 +676,37 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>พอร์ต 80</t>
+          <t>เซิร์ฟเวอร์จะเพิ่มประสิทธิภาพการส่งผ่านข้อมูลได้สองเท่า</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>พอร์ต 443</t>
+          <t>ผู้ดูแลระบบจะโดนตัดการเชื่อมต่อและโดนล็อกไม่ให้เข้าเซิร์ฟเวอร์ทันที</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>พอร์ต 22</t>
+          <t>หน้าจอระบบจะสั่งบังคับเปลี่ยนรหัสผ่านผู้ใช้อัตโนมัติ</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>พอร์ต 8006</t>
+          <t>ตัวบริการ Nginx Web Server จะปิดพอร์ต 80 เองถาวร</t>
         </is>
       </c>
       <c r="G5" s="10" t="n"/>
       <c r="H5" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J5" s="12" t="n"/>
     </row>
     <row r="6" ht="12.75" customHeight="1" s="17">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>หากต้องการเชื่อมต่อ SSH เข้าสู่เครื่องเซิร์ฟเวอร์ตู้เสมือนของตนเองด้วยสิทธิ์ root บนไอพี 192.168.10.150 ควรป้อนคำสั่งอย่างไร?</t>
+          <t>พอร์ตบริการใดต่อไปนี้ที่มีความสำคัญและจำเป็นต้องเปิดเพื่อใช้ควบคุมเซิร์ฟเวอร์ระยะไกลแบบปลอดภัย?</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
@@ -716,37 +716,37 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>ssh 192.168.10.150 -root</t>
+          <t>HTTP พอร์ต 80</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>ssh root@192.168.10.150</t>
+          <t>HTTPS พอร์ต 443</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>connect ssh root to 192.168.10.150</t>
+          <t>SSH พอร์ต 22</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>ssh root:192.168.10.150</t>
+          <t>MariaDB พอร์ต 3306</t>
         </is>
       </c>
       <c r="G6" s="14" t="n"/>
       <c r="H6" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J6" s="10" t="n"/>
     </row>
     <row r="7" ht="12.75" customHeight="1" s="17">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>ก่อนทำคำสั่งติดตั้ง Nginx บนระบบลินุกซ์ด้วยคำสั่ง sudo apt install nginx ข้อปฏิบัติข้อใดที่ระบบควรทำก่อนเสมอ?</t>
+          <t>หากต้องการกำหนดกฎอนุญาตการเข้าถึงพอร์ต 80 ของ Nginx บน UFW ควรป้อนคำสั่งอย่างไร?</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
@@ -756,27 +756,27 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>สั่งปิดพอร์ต 22 เพื่อรักษาความปลอดภัย</t>
+          <t>sudo ufw allow 80/tcp</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>รันคำสั่ง sudo apt update เพื่ออัปเดตรายการดัชนีแอปพลิเคชันล่าสุด</t>
+          <t>sudo ufw open port 80</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>สั่งลบโฟลเดอร์ผู้ใช้อื่นออกจากไดเรกทอรี /home</t>
+          <t>allow http on port 80</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>ทำการเปลี่ยนชื่อ Hostname เป็น nginx.local</t>
+          <t>sudo systemctl allow 80</t>
         </is>
       </c>
       <c r="G7" s="10" t="n"/>
       <c r="H7" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>25</v>
@@ -786,7 +786,7 @@
     <row r="8" ht="12.75" customHeight="1" s="17">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>คำสั่งใดที่ระบบใช้เพื่อเปิดให้ Nginx เริ่มต้นทำงานใหม่อีกครั้งทันทีแบบล้างโปรเซสทำงานเก่าหลังแก้ไขตัวแปร?</t>
+          <t>คำสั่งใดใช้เพื่อตรวจสอบสถานะ UFW แบบละเอียดพร้อมกฎการอนุญาตและปฏิเสธทั้งหมด?</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
@@ -796,37 +796,37 @@
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>sudo systemctl status nginx</t>
+          <t>sudo ufw show rules</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>sudo systemctl stop nginx</t>
+          <t>sudo ufw status verbose</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>sudo systemctl restart nginx</t>
+          <t>sudo ufw check status</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>sudo systemctl enable nginx</t>
+          <t>sudo systemctl status ufw</t>
         </is>
       </c>
       <c r="G8" s="14" t="n"/>
       <c r="H8" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="J8" s="10" t="n"/>
     </row>
     <row r="9" ht="12.75" customHeight="1" s="17">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>พิกัดโฟลเดอร์หรือไดเรกทอรีมาตรฐาน (Default Document Root) ที่ Nginx ใช้เก็บไฟล์หน้าเว็บ index.html คือพิกัดใด?</t>
+          <t>นโยบายค่าเริ่มต้น (Default Policy) ที่ปลอดภัยที่สุดในการตั้งค่า Inbound Firewall สำหรับเซิร์ฟเวอร์คือข้อใด?</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -836,37 +836,37 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>/etc/nginx/html/</t>
+          <t>บล็อกการเชื่อมต่อขาเข้าทั้งหมด ยกเว้นพอร์ตที่อนุญาต (Default Deny Inbound)</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>/var/www/html/</t>
+          <t>อนุญาตการเชื่อมต่อขาเข้าทั้งหมด ยกเว้นพอร์ตที่ระบุบล็อกไว้</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>/home/student/html/</t>
+          <t>อนุญาตการเชื่อมต่อทุกทิศทางโดยไม่มีการกรองเพื่อลดภาระของซีพียู</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>/usr/share/nginx/</t>
+          <t>ปิดกั้นการเชื่อมต่อขาออกทั้งหมดเพื่อป้องกันข้อมูลรั่วไหล</t>
         </is>
       </c>
       <c r="G9" s="14" t="n"/>
       <c r="H9" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J9" s="10" t="n"/>
     </row>
     <row r="10" ht="12.75" customHeight="1" s="17">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>เหตุใดการเขียนหรือลบไฟล์ index.html ในโฟลเดอร์ /var/www/html/ จึงจำเป็นต้องใช้คำสั่งนำหน้าด้วย sudo?</t>
+          <t>หากต้องการปฏิเสธ (Deny) ไม่ให้เครือข่ายภายนอกเชื่อมต่อเข้าพอร์ต MariaDB (3306) ควรใช้คำสั่งใด?</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
@@ -876,22 +876,22 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>เพราะโฟลเดอร์นี้ถูกรันด้วยสิทธิ์ความปลอดภัยสูงสุดและจำกัดสิทธิ์เฉพาะ root เท่านั้น</t>
+          <t>sudo ufw deny 3306/tcp</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>เพื่อทำให้หน้าเว็บเปิดแสดงผลกราฟิกสีสันได้รวดเร็วยิ่งขึ้น</t>
+          <t>sudo ufw close 3306</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>เพื่อหลีกเลี่ยงข้อจำกัดการเชื่อมต่อพอร์ต 8006</t>
+          <t>block port 3306 in firewall</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>เป็นกฎบังคับของการใช้บราวเซอร์ Google Chrome เสมอ</t>
+          <t>sudo ufw delete 3306</t>
         </is>
       </c>
       <c r="G10" s="14" t="n"/>
@@ -899,14 +899,14 @@
         <v>1</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="J10" s="10" t="n"/>
     </row>
     <row r="11" ht="12.75" customHeight="1" s="17">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>กฎเหล็กของแอดมินลินุกซ์ ในการตรวจสอบความถูกต้องของไวยากรณ์ในไฟล์ตั้งค่าของ Nginx ก่อนสั่งเริ่มระบบใหม่คือคำสั่งใด?</t>
+          <t>คำสั่ง 'sudo ufw status numbered' มีประโยชน์อย่างไรในการจัดการกฎไฟร์วอลล์?</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
@@ -916,22 +916,22 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>sudo systemctl test nginx</t>
+          <t>แสดงประวัติการเปลี่ยนแปลงกฎความปลอดภัยทั้งหมดพร้อมวันที่</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>sudo nginx -t</t>
+          <t>แสดงรายการกฎพร้อมตัวเลขลำดับเพื่อใช้ในการอ้างอิงตอนลบกฎ</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>check -nginx config</t>
+          <t>แสดงสถิติปริมาณแบนด์วิดท์ที่ผ่านในแต่ละกฎความปลอดภัย</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>verify nginx.conf</t>
+          <t>ตรวจสอบจำนวนครั้งที่เซิร์ฟเวอร์ทำการรีสตาร์ตระบบไฟร์วอลล์</t>
         </is>
       </c>
       <c r="G11" s="14" t="n"/>
@@ -939,14 +939,14 @@
         <v>2</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J11" s="10" t="n"/>
     </row>
     <row r="12" ht="12.75" customHeight="1" s="17">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>หากสั่งแก้ไขไฟล์คอนฟิกของ Nginx ผิดไวยากรณ์ไป 1 ตัวอักษร แล้วรันคำสั่ง restart บริการ ผลกระทบในข้อใดจะเกิดขึ้นกับเซิร์ฟเวอร์?</t>
+          <t>หากระบบไฟร์วอลล์ทำงานผิดพลาดหรือตั้งค่าพอร์ตสับสน และต้องการล้างกฎทั้งหมดกลับสู่ค่าเริ่มต้น ควรใช้คำสั่งใด?</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
@@ -956,22 +956,22 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>ระบบจะข้ามข้อความที่สะกดผิดไปรันค่าเดิมอัตโนมัติโดยไม่มีผลกระทบ</t>
+          <t>sudo ufw restart</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>บริการ Nginx จะล้มเหลวในการเปิดตัวและหยุดการทำงานลงทันที (เว็บล่ม)</t>
+          <t>sudo ufw reset</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>การ์ดเครือข่ายของเซิร์ฟเวอร์จะปิดตัวและยกเลิกรับค่า IP Address</t>
+          <t>sudo ufw delete all</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>หน้าจอเทอร์มินัลจะสั่งลบไฟล์เก็บข้อมูลเว็บทิ้งถาวร</t>
+          <t>sudo ufw clear rules</t>
         </is>
       </c>
       <c r="G12" s="14" t="n"/>
@@ -979,7 +979,7 @@
         <v>2</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="J12" s="10" t="n"/>
     </row>

</xml_diff>